<commit_message>
Actualiza registro semanal del Merval
</commit_message>
<xml_diff>
--- a/registro_merval.xlsx
+++ b/registro_merval.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR11"/>
+  <dimension ref="A1:CW11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -911,6 +911,31 @@
           <t>Semana 19 - Cierre</t>
         </is>
       </c>
+      <c r="CS1" t="inlineStr">
+        <is>
+          <t>Semana 20 - Fecha</t>
+        </is>
+      </c>
+      <c r="CT1" t="inlineStr">
+        <is>
+          <t>Semana 20 - Apertura</t>
+        </is>
+      </c>
+      <c r="CU1" t="inlineStr">
+        <is>
+          <t>Semana 20 - Máximo</t>
+        </is>
+      </c>
+      <c r="CV1" t="inlineStr">
+        <is>
+          <t>Semana 20 - Mínimo</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
+          <t>Semana 20 - Cierre</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1241,6 +1266,23 @@
       <c r="CR2" t="n">
         <v>7000</v>
       </c>
+      <c r="CS2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT2" t="n">
+        <v>6980</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>7015</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>6655</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>6685</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1571,6 +1613,23 @@
       <c r="CR3" s="1" t="n">
         <v>8835</v>
       </c>
+      <c r="CS3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT3" t="n">
+        <v>8880</v>
+      </c>
+      <c r="CU3" t="n">
+        <v>9220</v>
+      </c>
+      <c r="CV3" t="n">
+        <v>8605</v>
+      </c>
+      <c r="CW3" t="n">
+        <v>8760</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1901,6 +1960,23 @@
       <c r="CR4" s="1" t="n">
         <v>5525</v>
       </c>
+      <c r="CS4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT4" t="n">
+        <v>5505</v>
+      </c>
+      <c r="CU4" t="n">
+        <v>5640</v>
+      </c>
+      <c r="CV4" t="n">
+        <v>5190</v>
+      </c>
+      <c r="CW4" t="n">
+        <v>5215</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2231,6 +2307,23 @@
       <c r="CR5" t="n">
         <v>12420</v>
       </c>
+      <c r="CS5" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT5" t="n">
+        <v>12400</v>
+      </c>
+      <c r="CU5" t="n">
+        <v>12600</v>
+      </c>
+      <c r="CV5" t="n">
+        <v>11870</v>
+      </c>
+      <c r="CW5" t="n">
+        <v>12060</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2561,6 +2654,23 @@
       <c r="CR6" t="n">
         <v>668</v>
       </c>
+      <c r="CS6" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT6" t="n">
+        <v>670</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>680</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>648</v>
+      </c>
+      <c r="CW6" t="n">
+        <v>662</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2891,6 +3001,23 @@
       <c r="CR7" s="1" t="n">
         <v>871.5</v>
       </c>
+      <c r="CS7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT7" t="n">
+        <v>874.5</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>889</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>840</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>856.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3221,6 +3348,23 @@
       <c r="CR8" s="1" t="n">
         <v>2253</v>
       </c>
+      <c r="CS8" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT8" t="n">
+        <v>2240</v>
+      </c>
+      <c r="CU8" t="n">
+        <v>2313</v>
+      </c>
+      <c r="CV8" t="n">
+        <v>2055</v>
+      </c>
+      <c r="CW8" t="n">
+        <v>2078</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3551,6 +3695,23 @@
       <c r="CR9" s="1" t="n">
         <v>1954</v>
       </c>
+      <c r="CS9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT9" t="n">
+        <v>1950</v>
+      </c>
+      <c r="CU9" t="n">
+        <v>1970</v>
+      </c>
+      <c r="CV9" t="n">
+        <v>1870</v>
+      </c>
+      <c r="CW9" t="n">
+        <v>1881</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3881,6 +4042,23 @@
       <c r="CR10" t="n">
         <v>3120</v>
       </c>
+      <c r="CS10" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT10" t="n">
+        <v>3120</v>
+      </c>
+      <c r="CU10" t="n">
+        <v>3140</v>
+      </c>
+      <c r="CV10" t="n">
+        <v>2992.5</v>
+      </c>
+      <c r="CW10" t="n">
+        <v>3045</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4210,6 +4388,23 @@
       </c>
       <c r="CR11" s="1" t="n">
         <v>9515</v>
+      </c>
+      <c r="CS11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="CT11" t="n">
+        <v>9490</v>
+      </c>
+      <c r="CU11" t="n">
+        <v>9650</v>
+      </c>
+      <c r="CV11" t="n">
+        <v>9035</v>
+      </c>
+      <c r="CW11" t="n">
+        <v>9055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>